<commit_message>
Aula 13 conexao banco de dados
</commit_message>
<xml_diff>
--- a/Aula12/Alunos.xlsx
+++ b/Aula12/Alunos.xlsx
@@ -436,14 +436,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>jose</t>
+          <t>Jonas</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="C2" t="n">
-        <v>1.78</v>
+        <v>1.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>